<commit_message>
Add cards-case-study block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (9):
- blocks/cards-case-study/cards-case-study.css
- tools/importer/import-careers-overview.bundle.js
- tools/importer/import-careers-overview.js
- tools/importer/page-templates.json
- tools/importer/parsers/cards-case-study.js
- tools/importer/reports/en-us/careers.report.json
- tools/importer/reports/en-us/careers/experienced-professionals.report.json
- tools/importer/reports/en-us/careers/students.report.json
- tools/importer/reports/import-careers-overview.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-careers-overview.report.xlsx
+++ b/tools/importer/reports/import-careers-overview.report.xlsx
@@ -73,7 +73,7 @@
     <t>careers-overview</t>
   </si>
   <si>
-    <t>2026-09-11T08:23:32.141Z</t>
+    <t>2026-09-11T10:32:42.079Z</t>
   </si>
   <si>
     <t>Careers | Credera</t>
@@ -109,7 +109,7 @@
     <t>en-us/careers/experienced-professionals</t>
   </si>
   <si>
-    <t>2026-09-11T08:23:37.826Z</t>
+    <t>2026-09-11T10:32:48.434Z</t>
   </si>
   <si>
     <t>Experienced Professionals | Credera</t>
@@ -127,7 +127,7 @@
     <t>en-us/careers/students</t>
   </si>
   <si>
-    <t>2026-09-11T08:23:43.526Z</t>
+    <t>2026-09-11T10:32:55.181Z</t>
   </si>
   <si>
     <t>Students | Credera</t>

</xml_diff>

<commit_message>
careers_updated columns-feature block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (8):
- blocks/columns-feature/columns-feature.css
- tools/importer/import-careers-overview.bundle.js
- tools/importer/parsers/columns-feature.js
- tools/importer/reports/en-us/careers.report.json
- tools/importer/reports/en-us/careers/experienced-professionals.report.json
- tools/importer/reports/en-us/careers/students.report.json
- tools/importer/reports/import-careers-overview.report.xlsx
- tools/importer/transformers/credera-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-careers-overview.report.xlsx
+++ b/tools/importer/reports/import-careers-overview.report.xlsx
@@ -73,7 +73,7 @@
     <t>careers-overview</t>
   </si>
   <si>
-    <t>2026-09-14T05:45:21.793Z</t>
+    <t>2026-09-14T07:38:49.275Z</t>
   </si>
   <si>
     <t>Careers | Credera</t>
@@ -109,7 +109,7 @@
     <t>en-us/careers/experienced-professionals</t>
   </si>
   <si>
-    <t>2026-09-14T05:45:27.080Z</t>
+    <t>2026-09-14T07:38:55.025Z</t>
   </si>
   <si>
     <t>Experienced Professionals | Credera</t>
@@ -127,7 +127,7 @@
     <t>en-us/careers/students</t>
   </si>
   <si>
-    <t>2026-09-14T05:45:33.994Z</t>
+    <t>2026-09-14T07:39:01.626Z</t>
   </si>
   <si>
     <t>Students | Credera</t>

</xml_diff>

<commit_message>
Add cards-testimonial block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (18):
- blocks/cards-testimonial/README.md
- blocks/cards-testimonial/_cards-testimonial.json
- blocks/cards-testimonial/cards-testimonial.css
- blocks/cards-testimonial/cards-testimonial.js
- blocks/cards-testimonial/metadata.json
- component-definition.json
- component-filters.json
- component-models.json
- models/_section.json
- tools/importer/import-careers-overview.bundle.js
- tools/importer/import-careers-overview.js
- tools/importer/page-templates.json
- tools/importer/parsers/cards-testimonial.js
- tools/importer/reports/en-us/careers/experienced-professionals.report.json
- tools/importer/reports/en-us/careers/students.report.json
- tools/importer/reports/import-careers-overview.report.xlsx
- tools/importer/transformers/credera-cleanup.js
- tools/importer/urls-testimonial.txt
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-careers-overview.report.xlsx
+++ b/tools/importer/reports/import-careers-overview.report.xlsx
@@ -103,13 +103,13 @@
     <t>en-us/careers/experienced-professionals.report.json</t>
   </si>
   <si>
-    <t>["hero-home","columns-feature","columns-feature","columns-feature","cards-industry","cards-industry","hero-cta"]</t>
+    <t>["hero-home","columns-feature","columns-feature","columns-feature","cards-industry","cards-industry","cards-testimonial","hero-cta"]</t>
   </si>
   <si>
     <t>en-us/careers/experienced-professionals</t>
   </si>
   <si>
-    <t>2026-09-14T16:18:14.381Z</t>
+    <t>2026-09-15T04:54:05.960Z</t>
   </si>
   <si>
     <t>Experienced Professionals | Credera</t>
@@ -121,13 +121,13 @@
     <t>en-us/careers/students.report.json</t>
   </si>
   <si>
-    <t>["hero-home","columns-feature","cards-industry","hero-cta"]</t>
+    <t>["hero-home","columns-feature","cards-industry","cards-testimonial","hero-cta"]</t>
   </si>
   <si>
     <t>en-us/careers/students</t>
   </si>
   <si>
-    <t>2026-09-14T16:18:21.189Z</t>
+    <t>2026-09-15T04:54:11.428Z</t>
   </si>
   <si>
     <t>Students | Credera</t>

</xml_diff>

<commit_message>
Add cards-industry, faq blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (15):
- blocks/cards-industry/cards-industry.css
- blocks/faq/_faq.json
- blocks/faq/faq.css
- blocks/faq/faq.js
- component-definition.json
- component-filters.json
- component-models.json
- models/_section.json
- tools/importer/import-careers-overview.bundle.js
- tools/importer/import-careers-overview.js
- tools/importer/parsers/cards-industry.js
- tools/importer/reports/en-us/careers/experienced-professionals.report.json
- tools/importer/reports/en-us/careers/students.report.json
- tools/importer/reports/import-careers-overview.report.xlsx
- tools/importer/transformers/credera-faq.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-careers-overview.report.xlsx
+++ b/tools/importer/reports/import-careers-overview.report.xlsx
@@ -109,7 +109,7 @@
     <t>en-us/careers/experienced-professionals</t>
   </si>
   <si>
-    <t>2026-09-15T04:54:05.960Z</t>
+    <t>2026-09-15T06:17:40.088Z</t>
   </si>
   <si>
     <t>Experienced Professionals | Credera</t>
@@ -127,7 +127,7 @@
     <t>en-us/careers/students</t>
   </si>
   <si>
-    <t>2026-09-15T04:54:11.428Z</t>
+    <t>2026-09-15T06:17:45.783Z</t>
   </si>
   <si>
     <t>Students | Credera</t>

</xml_diff>

<commit_message>
Add hero-cta block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (7):
- blocks/hero-cta/hero-cta.css
- tools/importer/import-careers-overview.bundle.js
- tools/importer/parsers/hero-cta.js
- tools/importer/reports/en-us/careers.report.json
- tools/importer/reports/en-us/careers/experienced-professionals.report.json
- tools/importer/reports/en-us/careers/students.report.json
- tools/importer/reports/import-careers-overview.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-careers-overview.report.xlsx
+++ b/tools/importer/reports/import-careers-overview.report.xlsx
@@ -73,7 +73,7 @@
     <t>careers-overview</t>
   </si>
   <si>
-    <t>2026-09-14T16:18:08.115Z</t>
+    <t>2026-09-15T16:08:28.869Z</t>
   </si>
   <si>
     <t>Careers | Credera</t>
@@ -109,7 +109,7 @@
     <t>en-us/careers/experienced-professionals</t>
   </si>
   <si>
-    <t>2026-09-15T06:17:40.088Z</t>
+    <t>2026-09-15T16:07:02.547Z</t>
   </si>
   <si>
     <t>Experienced Professionals | Credera</t>
@@ -127,7 +127,7 @@
     <t>en-us/careers/students</t>
   </si>
   <si>
-    <t>2026-09-15T06:17:45.783Z</t>
+    <t>2026-09-15T16:07:08.782Z</t>
   </si>
   <si>
     <t>Students | Credera</t>

</xml_diff>

<commit_message>
Add hero-home block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (7):
- blocks/hero-home/hero-home.css
- tools/importer/import-careers-overview.bundle.js
- tools/importer/parsers/hero-home.js
- tools/importer/reports/en-us/careers/experienced-professionals.report.json
- tools/importer/reports/en-us/careers/students.report.json
- tools/importer/reports/import-careers-overview.report.xlsx
- tools/importer/transformers/credera-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-careers-overview.report.xlsx
+++ b/tools/importer/reports/import-careers-overview.report.xlsx
@@ -109,7 +109,7 @@
     <t>en-us/careers/experienced-professionals</t>
   </si>
   <si>
-    <t>2026-09-15T16:07:02.547Z</t>
+    <t>2026-09-15T20:02:25.667Z</t>
   </si>
   <si>
     <t>Experienced Professionals | Credera</t>
@@ -127,7 +127,7 @@
     <t>en-us/careers/students</t>
   </si>
   <si>
-    <t>2026-09-15T16:07:08.782Z</t>
+    <t>2026-09-15T20:02:32.127Z</t>
   </si>
   <si>
     <t>Students | Credera</t>

</xml_diff>

<commit_message>
Update importer for video duplication issue
Automated migration updates generated by Experience Modernization Agent.

Changed files (5):
- tools/importer/import-careers-overview.bundle.js
- tools/importer/reports/en-us/careers/experienced-professionals.report.json
- tools/importer/reports/en-us/careers/students.report.json
- tools/importer/reports/import-careers-overview.report.xlsx
- tools/importer/transformers/credera-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-careers-overview.report.xlsx
+++ b/tools/importer/reports/import-careers-overview.report.xlsx
@@ -109,7 +109,7 @@
     <t>en-us/careers/experienced-professionals</t>
   </si>
   <si>
-    <t>2026-09-15T20:02:25.667Z</t>
+    <t>2026-09-15T20:56:42.640Z</t>
   </si>
   <si>
     <t>Experienced Professionals | Credera</t>
@@ -127,7 +127,7 @@
     <t>en-us/careers/students</t>
   </si>
   <si>
-    <t>2026-09-15T20:02:32.127Z</t>
+    <t>2026-09-15T20:56:48.182Z</t>
   </si>
   <si>
     <t>Students | Credera</t>

</xml_diff>

<commit_message>
Add cards-industry block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (15):
- blocks/cards-industry/cards-industry.css
- blocks/cards-industry/cards-industry.js
- icons/team-ai-data.png
- icons/team-business-enablement.svg
- icons/team-digital-solutions.svg
- icons/team-experience-design.svg
- icons/team-management-consulting.svg
- icons/team-marketing-technology.svg
- icons/team-technology-solutions.svg
- tools/importer/import-careers-overview.bundle.js
- tools/importer/import-careers-overview.js
- tools/importer/parsers/cards-industry.js
- tools/importer/reports/en-us/careers/experienced-professionals.report.json
- tools/importer/reports/en-us/careers/students.report.json
- tools/importer/reports/import-careers-overview.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-careers-overview.report.xlsx
+++ b/tools/importer/reports/import-careers-overview.report.xlsx
@@ -109,7 +109,7 @@
     <t>en-us/careers/experienced-professionals</t>
   </si>
   <si>
-    <t>2026-09-15T20:56:42.640Z</t>
+    <t>2026-09-15T21:32:41.718Z</t>
   </si>
   <si>
     <t>Experienced Professionals | Credera</t>
@@ -127,7 +127,7 @@
     <t>en-us/careers/students</t>
   </si>
   <si>
-    <t>2026-09-15T20:56:48.182Z</t>
+    <t>2026-09-15T21:32:48.135Z</t>
   </si>
   <si>
     <t>Students | Credera</t>

</xml_diff>

<commit_message>
Fix columns-feature callout variant sync to AEM
- Add name+model to columns-feature xwalk template so md2jcr resolves the
  model and its classes field (variant classes were silently dropped for the
  native columns component, affecting both featured and callout callouts).
- Use single-word variant tokens (callout, featured) that survive the
  html2md->md2jcr round-trip intact; multi-word/hyphenated tokens get
  corrupted into broken class names.
- Rename card-callout CSS variant to callout; re-import careers pages.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-careers-overview.report.xlsx
+++ b/tools/importer/reports/import-careers-overview.report.xlsx
@@ -73,7 +73,7 @@
     <t>careers-overview</t>
   </si>
   <si>
-    <t>2026-09-15T16:08:28.869Z</t>
+    <t>2026-09-16T15:40:24.607Z</t>
   </si>
   <si>
     <t>Careers | Credera</t>
@@ -109,7 +109,7 @@
     <t>en-us/careers/experienced-professionals</t>
   </si>
   <si>
-    <t>2026-09-16T13:03:56.137Z</t>
+    <t>2026-09-16T15:40:31.127Z</t>
   </si>
   <si>
     <t>Experienced Professionals | Credera</t>
@@ -127,7 +127,7 @@
     <t>en-us/careers/students</t>
   </si>
   <si>
-    <t>2026-09-15T21:32:48.135Z</t>
+    <t>2026-09-16T15:40:37.941Z</t>
   </si>
   <si>
     <t>Students | Credera</t>

</xml_diff>